<commit_message>
Rename PID structure type
</commit_message>
<xml_diff>
--- a/Docs/Injectors Lag.xlsx
+++ b/Docs/Injectors Lag.xlsx
@@ -36,7 +36,7 @@
     <t>Bosch 0280155746 200cc</t>
   </si>
   <si>
-    <t>Bosch 0280155968 420cc</t>
+    <t>Bosch 0280158235 731cc</t>
   </si>
 </sst>
 </file>
@@ -553,11 +553,15 @@
         <f>H3-I3</f>
         <v>1.8599999999999999</v>
       </c>
-      <c r="K3" s="1"/>
-      <c r="L3" s="2"/>
+      <c r="K3" s="1">
+        <v>4.1399999999999997</v>
+      </c>
+      <c r="L3" s="9">
+        <v>0.7</v>
+      </c>
       <c r="M3" s="3">
         <f>K3-L3</f>
-        <v>0</v>
+        <v>3.4399999999999995</v>
       </c>
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.25">
@@ -594,11 +598,15 @@
         <f t="shared" ref="J4:J8" si="2">H4-I4</f>
         <v>1.08</v>
       </c>
-      <c r="K4" s="1"/>
-      <c r="L4" s="2"/>
+      <c r="K4" s="1">
+        <v>2.44</v>
+      </c>
+      <c r="L4" s="9">
+        <v>0.7</v>
+      </c>
       <c r="M4" s="3">
         <f t="shared" ref="M4:M8" si="3">K4-L4</f>
-        <v>0</v>
+        <v>1.74</v>
       </c>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.25">
@@ -635,11 +643,15 @@
         <f t="shared" si="2"/>
         <v>0.77000000000000013</v>
       </c>
-      <c r="K5" s="1"/>
-      <c r="L5" s="2"/>
+      <c r="K5" s="1">
+        <v>1.84</v>
+      </c>
+      <c r="L5" s="9">
+        <v>0.7</v>
+      </c>
       <c r="M5" s="3">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>1.1400000000000001</v>
       </c>
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.25">
@@ -676,11 +688,15 @@
         <f t="shared" si="2"/>
         <v>0.46000000000000008</v>
       </c>
-      <c r="K6" s="1"/>
-      <c r="L6" s="2"/>
+      <c r="K6" s="1">
+        <v>1.5</v>
+      </c>
+      <c r="L6" s="9">
+        <v>0.7</v>
+      </c>
       <c r="M6" s="3">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.25">
@@ -717,11 +733,15 @@
         <f t="shared" si="2"/>
         <v>0.28999999999999992</v>
       </c>
-      <c r="K7" s="1"/>
-      <c r="L7" s="2"/>
+      <c r="K7" s="1">
+        <v>1.28</v>
+      </c>
+      <c r="L7" s="9">
+        <v>0.74</v>
+      </c>
       <c r="M7" s="3">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>0.54</v>
       </c>
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.25">
@@ -758,11 +778,15 @@
         <f t="shared" si="2"/>
         <v>0.10999999999999999</v>
       </c>
-      <c r="K8" s="4"/>
-      <c r="L8" s="5"/>
+      <c r="K8" s="4">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="L8" s="5">
+        <v>0.8</v>
+      </c>
       <c r="M8" s="6">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>0.30000000000000004</v>
       </c>
     </row>
   </sheetData>

</xml_diff>